<commit_message>
🤖 Post-Match: Storico validato e archiviato senza doppioni
</commit_message>
<xml_diff>
--- a/Database_Storico_Completo.xlsx
+++ b/Database_Storico_Completo.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -878,6 +878,149 @@
         </is>
       </c>
       <c r="AE3" t="inlineStr">
+        <is>
+          <t>PERDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FIFA World Cup</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>17/06/2026 22:00</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>England - Croatia</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0-1 MG</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0-1 MG</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>1X</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>OVER 1.5</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>UNDER 2.5</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>UNDER 3.5</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>NOGOAL</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>1X+UNDER</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Non disponibile</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>VINCENTE</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>PERDENTE</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>VINCENTE</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>PERDENTE</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>VINCENTE</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>PERDENTE</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>PERDENTE</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>PERDENTE</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>PERDENTE</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>In attesa</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
         <is>
           <t>PERDENTE</t>
         </is>

</xml_diff>